<commit_message>
Remove outdated sidebar navigation and update pipeline scripts; delete unused data files related to tourism statistics.
</commit_message>
<xml_diff>
--- a/data/raw/Gab_Data_Wisman_Bali.xlsx
+++ b/data/raw/Gab_Data_Wisman_Bali.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gessya\colyfe\Semester 7\Skripsi\Data\Wisman Bali\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Kuliah\6th semester\DSP\MultiMetode\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62195A5D-BEE5-457E-9E30-503E1E2824AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95A0307-97C9-4C54-8D55-F859DCB028F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F8BD8DBD-627C-4707-8C9A-45E3D0756ED3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8BD8DBD-627C-4707-8C9A-45E3D0756ED3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,9 +74,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -392,7 +394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69FC4C4B-999C-42CD-B8E8-AD2533F4A612}">
-  <dimension ref="A1:B193"/>
+  <dimension ref="A1:B209"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -1939,6 +1941,134 @@
         <v>551100</v>
       </c>
     </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A194" s="1">
+        <v>45658</v>
+      </c>
+      <c r="B194" s="2">
+        <v>529897</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A195" s="1">
+        <v>45689</v>
+      </c>
+      <c r="B195" s="2">
+        <v>450697</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A196" s="1">
+        <v>45717</v>
+      </c>
+      <c r="B196" s="2">
+        <v>470851</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A197" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B197" s="2">
+        <v>591221</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A198" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B198" s="2">
+        <v>602213</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A199" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B199" s="2">
+        <v>637868</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A200" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B200" s="2">
+        <v>697107</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A201" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B201" s="2">
+        <v>682866</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A202" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B202" s="2">
+        <v>635149</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A203" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B203" s="2">
+        <v>594853</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A204" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B204" s="2">
+        <v>483364</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A205" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B205" s="2">
+        <v>572668</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A206" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B206" s="3">
+        <v>502205</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A207" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B207" s="3">
+        <v>492289</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A208" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B208" s="3">
+        <v>472070</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A209" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B209" s="3">
+        <v>553328</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>